<commit_message>
warning wave table update
</commit_message>
<xml_diff>
--- a/Table/car_survivor_tables.xlsx
+++ b/Table/car_survivor_tables.xlsx
@@ -20,6 +20,7 @@
     <sheet name="TB_LangLevelUpSelect_des" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="TB_Stage" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="Sheet1" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="TB_WarningWave" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1319,7 +1320,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.9"/>
   <sheetData>
     <row r="1">
@@ -1368,6 +1369,11 @@
           <t>arena_radius</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>ww_group_id</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1407,7 +1413,12 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>20</v>
+        <v>50</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>WW_CH1_1</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -1448,7 +1459,12 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>20</v>
+        <v>50</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>WW_CH1_2</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -1489,7 +1505,12 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>20</v>
+        <v>50</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>WW_CH1_3</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1508,6 +1529,522 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.9"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ww_group_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>wave_no</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>mon_id</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>spawn_count</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>spawn_interval</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>max_enemies</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>difficulty_scale</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>start_time</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>WW_CH1_1</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>MON_001</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>초반 웨이브</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>WW_CH1_1</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>MON_002</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F3" t="n">
+        <v>60</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H3" t="n">
+        <v>10</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>10초 후 추가</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>WW_CH1_1</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>MON_003</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>80</v>
+      </c>
+      <c r="G4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H4" t="n">
+        <v>20</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>20초 후 강화</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>WW_CH1_1</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>MON_001</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F5" t="n">
+        <v>80</v>
+      </c>
+      <c r="G5" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H5" t="n">
+        <v>30</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>30초 후 가속</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>WW_CH1_1</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>MON_004</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F6" t="n">
+        <v>100</v>
+      </c>
+      <c r="G6" t="n">
+        <v>4</v>
+      </c>
+      <c r="H6" t="n">
+        <v>45</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>45초 후 폭풍</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>WW_CH1_2</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>MON_002</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F7" t="n">
+        <v>60</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Stage2 초반</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>WW_CH1_2</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MON_003</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>70</v>
+      </c>
+      <c r="G8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" t="n">
+        <v>10</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>10초 후</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>WW_CH1_2</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MON_004</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>6</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F9" t="n">
+        <v>90</v>
+      </c>
+      <c r="G9" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H9" t="n">
+        <v>20</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>20초 후</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>WW_CH1_2</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>MON_001</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>8</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G10" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H10" t="n">
+        <v>35</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>35초 후 폭풍</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>WW_CH1_3</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>MON_003</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>5</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>70</v>
+      </c>
+      <c r="G11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Stage3 초반</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>WW_CH1_3</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>MON_004</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>6</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F12" t="n">
+        <v>80</v>
+      </c>
+      <c r="G12" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H12" t="n">
+        <v>10</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>10초 후</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>WW_CH1_3</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>MON_001</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>8</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F13" t="n">
+        <v>90</v>
+      </c>
+      <c r="G13" t="n">
+        <v>4</v>
+      </c>
+      <c r="H13" t="n">
+        <v>20</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>20초 후</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>WW_CH1_3</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>4</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>MON_002</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>10</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F14" t="n">
+        <v>100</v>
+      </c>
+      <c r="G14" t="n">
+        <v>5</v>
+      </c>
+      <c r="H14" t="n">
+        <v>30</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>30초 후 최종</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 

</xml_diff>